<commit_message>
Search only hotels: drop sanatorium-type markers, reject institutions, remove hygiene kits
- Keywords file: markers limited to hotels/гостиницы; sanatoriums, pansionats, rest bases,
  dormitories, schools, social and state/municipal institutions become strong minus words;
  hygiene kits category, its codes and queries removed; generic keys need a hotel marker
- Classifier: minus words from a customer name that carries a hotel marker are ignored
  (departmental hotels such as FGBU hotel complexes stay relevant)
- Startup applies a changed project keyword file unless a file was uploaded manually

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SPYFSXLy6BMw3QpJjiagSA
</commit_message>
<xml_diff>
--- a/Velmorium_ключевые_слова_тендеры.xlsx
+++ b/Velmorium_ключевые_слова_тендеры.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товарные ключи" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Маркеры заказчика" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Минус-слова" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Коды ОКПД2-КТРУ" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Готовые запросы" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Площадки" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Товарные ключи" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Маркеры заказчика" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Минус-слова" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Коды ОКПД2-КТРУ" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Готовые запросы" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Площадки" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Товарные ключи'!$A$1:$F$88</definedName>
@@ -578,7 +578,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Одноразовые гигиенические наборы: зубной, бритвенный, гигиенический (ватные палочки, диски, пилочка)</t>
+          <t>• Одноразовые гигиенические наборы: зубной, бритвенный, гигиенический (ватные палочки, диски, пилочка) — в поиске тендеров не используются (решение 22.10.2026)</t>
         </is>
       </c>
     </row>
@@ -654,14 +654,14 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Маркеры заказчика — слова в названии заказчика, предмете закупки или месте поставки, указывающие на отель/санаторий.</t>
+          <t>Маркеры заказчика — слова в названии заказчика, предмете закупки или месте поставки, указывающие на отель или гостиницу (санатории, пансионаты и базы отдыха не ищем).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Минус-слова — исключают нерелевантные закупки (медицина, соцучреждения, услуги прачечной, спецодежда).</t>
+          <t>Минус-слова — исключают нерелевантные закупки (медицина, соцучреждения, санатории, учреждения, услуги прачечной, спецодежда).</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>халат* (гост*|бассейн*|спа)</t>
+          <t>халат* для гост* | халат* (бассейн*|спа)</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E47" s="5" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E54" s="5" t="n">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Самодостаточный</t>
+          <t>Нужен маркер</t>
         </is>
       </c>
       <c r="E68" s="5" t="n">
@@ -2794,370 +2794,90 @@
       <c r="F75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>одноразовые гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>одноразов* гигиен* набор*</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F76" s="5" t="inlineStr"/>
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>Смежное (нет на сайте)</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>шторы / портьеры / тюль / блэкаут</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>штор* | портьер* | тюл* | блэкаут* | blackout</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Нужен маркер</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>Часто в одном лоте при оснащении номеров</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>гостевая косметика / гостиничная косметика</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>гостев* косметик* | гостиничн* косметик*</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F77" s="5" t="inlineStr"/>
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>Смежное (нет на сайте)</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>столовое бельё / скатерти / салфетки столовые</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>столов* бель* | скатерт* | салфетк* столов*</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Нужен маркер</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Ресторан при отеле</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>косметика для гостиниц / отелей</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>косметик* для (гостиниц*|отел*)</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F78" s="5" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>одноразовые принадлежности для гостиниц</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>одноразов* принадлежн*</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F79" s="5" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>amenities / эмэнитис</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>amenities | эмэнит* | аменит*</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>Отраслевой термин</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>зубной набор</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>зубн* набор*</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>Есть в ассортименте</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>бритвенный набор</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>бритвен* набор*</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Есть в ассортименте</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>гигиенический набор / ватные палочки и диски</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>гигиен* набор* | ватн* (палоч*|диск*)</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>Смежное (нет на сайте)</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>мольтон / наскатертник</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>мольтон* | наскатертник*</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>Нужен маркер</t>
         </is>
       </c>
-      <c r="E83" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
-          <t>Есть в ассортименте</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>индивидуальные средства гигиены / мыло одноразовое / шампунь во флаконах</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="inlineStr">
-        <is>
-          <t>индивидуальн* средств* гигиен* | мыл* одноразов* | шампун*</t>
-        </is>
-      </c>
-      <c r="D84" s="6" t="inlineStr">
-        <is>
-          <t>Нужен маркер</t>
-        </is>
-      </c>
-      <c r="E84" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F84" s="6" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>шапочка для душа / швейный набор / набор для обуви</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="inlineStr">
-        <is>
-          <t>шапочк* для душ* | швейн* набор* | набор* для обув*</t>
-        </is>
-      </c>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>Самодостаточный</t>
-        </is>
-      </c>
-      <c r="E85" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F85" s="6" t="inlineStr">
-        <is>
-          <t>Классический гостевой ассортимент</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>Смежное (нет на сайте)</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
-        <is>
-          <t>шторы / портьеры / тюль / блэкаут</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>штор* | портьер* | тюл* | блэкаут* | blackout</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>Нужен маркер</t>
-        </is>
-      </c>
-      <c r="E86" s="7" t="n">
+      <c r="E78" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>Часто в одном лоте при оснащении номеров</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="7" t="inlineStr">
-        <is>
-          <t>Смежное (нет на сайте)</t>
-        </is>
-      </c>
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>столовое бельё / скатерти / салфетки столовые</t>
-        </is>
-      </c>
-      <c r="C87" s="7" t="inlineStr">
-        <is>
-          <t>столов* бель* | скатерт* | салфетк* столов*</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>Нужен маркер</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>Ресторан при отеле</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t>Смежное (нет на сайте)</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
-        <is>
-          <t>мольтон / наскатертник</t>
-        </is>
-      </c>
-      <c r="C88" s="7" t="inlineStr">
-        <is>
-          <t>мольтон* | наскатертник*</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>Нужен маркер</t>
-        </is>
-      </c>
-      <c r="E88" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F88" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F88"/>
@@ -3171,7 +2891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3221,7 +2941,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>гостиниц*</t>
+          <t>гостиниц* | гостиничн*</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
@@ -3371,12 +3091,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>санаторий / санаторно-курортный</t>
+          <t>резорт / resort</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>санатори* | санаторно-курорт*</t>
+          <t>резорт* | resort</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
@@ -3384,7 +3104,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Крупнейший сегмент госзакупок «гостиничного» текстиля</t>
+          <t>Только «резорт» — курорты и санатории не ищем</t>
         </is>
       </c>
     </row>
@@ -3396,12 +3116,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>пансионат</t>
+          <t>загородный отель / парк-отель</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>пансионат*</t>
+          <t>загородн* отел* | парк-отел*</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
@@ -3410,25 +3130,25 @@
       <c r="E10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Тип заказчика</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>дом отдыха</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>дом* отдых*</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5" t="inlineStr"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>глэмпинг / эко-отель</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>глэмпинг* | глемпинг* | эко-отел*</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -3438,60 +3158,68 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>профилакторий</t>
+          <t>спа-отель</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>профилактори*</t>
+          <t>спа-отел* | spa-отел* | spa hotel</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Не искать «спа» без дефиса — ловит «спасательный» и т.п.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Тип заказчика</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>курорт / курортный комплекс / резорт</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>курорт* | резорт* | resort</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5" t="inlineStr"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>гостевая резиденция / дом приёмов</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>резиденц* | дом* при[её]м*</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Ведомственные объекты</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Тип заказчика</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>база отдыха / турбаза / туристический комплекс</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>баз* отдых* | турбаз* | туристическ* комплекс*</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ведомственная гостиница / гостиница при вузе</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>ведомствен* гостиниц*</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -3501,12 +3229,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>оздоровительный комплекс / центр</t>
+          <t>hotel / inn / suites</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>оздоровительн* (комплекс*|центр*)</t>
+          <t>hotel | inn | suites</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -3514,66 +3242,74 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Может быть детский лагерь — проверять</t>
+          <t>Название заказчика на коммерческих площадках</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Тип заказчика</t>
+          <t>Контекст закупки</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>загородный клуб / загородный отель / парк-отель</t>
+          <t>номерной фонд / номера</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>загородн* (клуб*|отел*) | парк-отел*</t>
+          <t>номерн* фонд* | для номер*</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Сильный сигнал в предмете закупки или ТЗ</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Тип заказчика</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>глэмпинг / кемпинг / эко-отель</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>глэмпинг* | глемпинг* | кемпинг* | эко-отел*</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="6" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Контекст закупки</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>для проживания гостей / для гостей</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>проживан* гост* | для гост*</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>«проживание» без «гостей» — и общежития</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Тип заказчика</t>
+          <t>Контекст закупки</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>спа-отель / SPA-комплекс / термальный комплекс</t>
+          <t>открытие отеля / реновация / ребрендинг номеров</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>спа-* | spa | термальн*</t>
+          <t>открыт* отел* | реновац* номер* | ребрендинг* номер*</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -3581,318 +3317,30 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Не искать «спа» без дефиса — ловит «спасательный» и т.п.</t>
+          <t>Крупные комплексные лоты</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Тип заказчика</t>
+          <t>Контекст закупки</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>гостевая резиденция / дом приёмов</t>
+          <t>хаускипинг / горничные / служба размещения</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>резиденц* | дом* при[её]м*</t>
+          <t>хаускипинг* | housekeeping | горничн* | служб* размещен*</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Ведомственные объекты</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Тип заказчика</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>ведомственная гостиница / гостиница при вузе</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>ведомствен* гостиниц*</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Тип заказчика</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>общежитие / общежитие гостиничного типа</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>общежити*</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Похожий ассортимент, но ниже чек; включать по желанию</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Тип заказчика</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>hotel / inn / suites</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>hotel | inn | suites</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Название заказчика на коммерческих площадках</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>номерной фонд / номера</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>номерн* фонд* | для номер*</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Сильный сигнал в предмете закупки или ТЗ</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>для проживания гостей / для гостей</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>проживан* | для гост*</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>открытие отеля / реновация / ребрендинг номеров</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>открыт* отел* | реновац* | ребрендинг*</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Крупные комплексные лоты</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>хаускипинг / горничные / служба размещения</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>хаускипинг* | housekeeping | горничн* | служб* размещен*</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>брендирование / вышивка логотипа</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>брендир* | вышивк* логотип* | вышивк*</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Чаще всего в гостиничных ТЗ</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Контекст закупки</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>промышленная стирка / выдерживает 200+ стирок</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>промышленн* стирк*</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Требование гостиничного/ресторанного текстиля</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Группы заказчиков (ориентиры)</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>РЖД-Здоровье (санатории)</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>ржд-здоровье</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Сеть санаториев; проверить актуальность названия</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Группы заказчиков (ориентиры)</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Управление делами Президента (санатории, гостиницы)</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>управлени* делами президент*</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>ФГБУ санатории и гостиничные комплексы</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Группы заказчиков (ориентиры)</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Санаторно-курортные комплексы Минобороны, МВД, ФМБА, профсоюзов</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>санаторно-курортн* комплекс*</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E31"/>
@@ -3906,7 +3354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3987,11 +3435,7 @@
           <t>Сильный</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Санатории с медпрофилем пишут «санаторий» — маркер заказчика их вернёт</t>
-        </is>
-      </c>
+      <c r="E3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -4153,14 +3597,10 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Средний</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Санатории-интернаты — проверять вручную</t>
-        </is>
-      </c>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -4253,14 +3693,10 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Средний</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Но санатории Минобороны — релевантны</t>
-        </is>
-      </c>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -4515,6 +3951,179 @@
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Санатории и отдых (не отели)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>санаторий / пансионат / профилакторий / дом и база отдыха</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>санатори* | санаторно-курорт* | пансионат* | профилактори* | дом* отдых* | баз* отдых* | турбаз*</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Нужны только отели и гостиницы. «Гостиница санатория» — маркер вернёт «на проверку»</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Санатории и отдых (не отели)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>детский лагерь / оздоровительный центр</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>лагер* | оздоровительн*</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Образование / соцсфера</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>общежитие</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>общежити*</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Образование / соцсфера</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>колледж / техникум / университет / институт</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>колледж* | техникум* | университет* | институт* | вуз*</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Гостиница при вузе с маркером в названии заказчика останется релевантной</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Образование / соцсфера</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>социальное учреждение / реабилитация</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>социальн* | реабилитац*</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Учреждения</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>государственное / муниципальное учреждение</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>учреждени* | гбу | мбу | гку | мку | гау | мау | фгбу | фгку | фгау | фку | гбуз | гауз | гбоу | мбоу | мадоу | гбпоу | фгбоу</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Сильный</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Нужны только отели. Если в названии заказчика-учреждения есть «гостиница/отель» — он остаётся релевантным (ведомственные гостиницы)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Учреждения</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>администрация / министерство / управление</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>администрац* | министерств* | управлени* | департамент*</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E24"/>
@@ -4528,7 +4137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5148,39 +4757,35 @@
       <c r="F22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>20.42</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>13.92.15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>ОКПД2</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Духи и косметические средства (группа)</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Ориентир; подкоды зависят от состава набора</t>
-        </is>
-      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Занавеси и шторы для интерьеров</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Смежное: шторы</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>32.91.11</t>
+          <t>13.92.13</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -5190,74 +4795,18 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Мётлы и щётки (вкл. зубные щётки)</t>
+          <t>Бельё столовое</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Зубной набор</t>
+          <t>Смежное: скатерти</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Ориентир</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>13.92.15</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>ОКПД2</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Занавеси и шторы для интерьеров</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Смежное: шторы</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>13.92.13</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>ОКПД2</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Бельё столовое</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Смежное: скатерти</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F26"/>
@@ -5271,7 +4820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5425,7 +4974,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>гостиничная косметика</t>
+          <t>топпер</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr"/>
@@ -5438,7 +4987,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>одноразовые принадлежности для гостиниц</t>
+          <t>страйп-сатин</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr"/>
@@ -5451,7 +5000,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>топпер</t>
+          <t>оснащение номерного фонда</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr"/>
@@ -5459,165 +5008,83 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Без логики (фраза)</t>
+          <t>Булев (агрегаторы)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>страйп-сатин</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr"/>
+          <t>(гостиниц* | гостиничн* | отел* | хостел* | "гостевой дом" | апарт-отел*) &amp; ("мягкий инвентарь" | "постельное белье" | полотенц* | халат* | тапоч* | подушк* | одеял* | наматрасник* | покрывал*) -медицин* -больниц* -санатори* -аренд* -детск*</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Основной запрос. Синтаксис операторов адаптировать под площадку</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Без логики (фраза)</t>
+          <t>Булев (агрегаторы)</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>оснащение номерного фонда</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr"/>
+          <t>(гостиничн* | "для гостиниц*" | "для отел*") &amp; (текстил* | бель* | полотенц* | халат* | тапоч*)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Самодостаточные фразы</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Без логики (фраза)</t>
+          <t>Булев (агрегаторы)</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>мягкий инвентарь санаторий</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr"/>
+          <t>("страйп-сатин" | "страйп сатин" | полисатин | поликоттон | топпер*) -медицин*</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Сигнальные ткани/товары</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Без логики (фраза)</t>
+          <t>Фильтр по коду</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>постельное белье санаторий</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr"/>
+          <t>ОКПД2 13.92.12 + регион/заказчик с маркером из листа «Маркеры заказчика»</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>ЕИС, Контур.Закупки и др. — фильтр по коду + слово в названии заказчика</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Без логики (фраза)</t>
+          <t>Фильтр по коду</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>мягкий инвентарь пансионат</t>
+          <t>ОКПД2 13.92.14, 13.92.24, 13.92.11, 14.14.22, 15.20.14 + маркер заказчика (отель/гостиница)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Булев (агрегаторы)</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>(гостиниц* | отел* | хостел* | санатори* | пансионат* | "дом отдыха" | "база отдыха" | курорт*) &amp; ("мягкий инвентарь" | "постельное белье" | полотенц* | халат* | тапоч* | подушк* | одеял* | наматрасник* | покрывал*) -медицин* -больниц* -аренд* -детск*</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Основной запрос. Синтаксис операторов адаптировать под площадку</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Булев (агрегаторы)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>(гостиничн* | "для гостиниц*" | "для отел*") &amp; (текстил* | бель* | полотенц* | халат* | тапоч* | косметик*)</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Самодостаточные фразы</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Булев (агрегаторы)</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>("страйп-сатин" | "страйп сатин" | полисатин | поликоттон | топпер*) -медицин*</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Сигнальные ткани/товары</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Булев (агрегаторы)</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>(одноразов* | гостев* | гостиничн*) &amp; ("гигиенический набор" | "зубной набор" | "бритвенный набор" | косметик* | amenities)</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Гигиенические наборы</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Фильтр по коду</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ОКПД2 13.92.12 + регион/заказчик с маркером из листа «Маркеры заказчика»</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>ЕИС, Контур.Закупки и др. — фильтр по коду + слово в названии заказчика</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Фильтр по коду</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>ОКПД2 13.92.14, 13.92.24, 13.92.11, 14.14.22, 15.20.14 + маркер заказчика</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:C24"/>

</xml_diff>